<commit_message>
fixing old code with the student schema updates
</commit_message>
<xml_diff>
--- a/data/students.xlsx
+++ b/data/students.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahmed\OneDrive\Bureau\isamm-student-managment-platform\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahmed\OneDrive\Bureau\Projects\isamm-student-managment-platform\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C47994D9-B6B7-48A0-8B05-34DDE6DDB400}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1DFCFCC-7231-40B0-AB5E-E31B76A902CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5625" yWindow="2745" windowWidth="19695" windowHeight="11505" xr2:uid="{AFD31129-8B99-4084-8265-242CB6D304A0}"/>
+    <workbookView xWindow="5085" yWindow="3705" windowWidth="21600" windowHeight="11505" xr2:uid="{AFD31129-8B99-4084-8265-242CB6D304A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="28">
   <si>
     <t>firstName</t>
   </si>
@@ -56,12 +56,6 @@
     <t>phone</t>
   </si>
   <si>
-    <t>cv</t>
-  </si>
-  <si>
-    <t>fieldOfStudy</t>
-  </si>
-  <si>
     <t>level</t>
   </si>
   <si>
@@ -86,21 +80,6 @@
     <t>Ghazi</t>
   </si>
   <si>
-    <t>Chiraz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oumaima </t>
-  </si>
-  <si>
-    <t>Ilyes</t>
-  </si>
-  <si>
-    <t>hafsi</t>
-  </si>
-  <si>
-    <t>ben boubaker</t>
-  </si>
-  <si>
     <t>nefzi</t>
   </si>
   <si>
@@ -116,73 +95,31 @@
     <t>ben Ali</t>
   </si>
   <si>
-    <t>ahmed_cv.pdf</t>
-  </si>
-  <si>
-    <t>ali_cv.pdf</t>
-  </si>
-  <si>
-    <t>amine_cv.pdf</t>
-  </si>
-  <si>
-    <t>amira_cv.pdf</t>
-  </si>
-  <si>
-    <t>islem_cv.pdf</t>
-  </si>
-  <si>
-    <t>ghazi_cv.pdf</t>
-  </si>
-  <si>
-    <t>chiraz_cv.pdf</t>
-  </si>
-  <si>
-    <t>oumaima_cv.pdf</t>
-  </si>
-  <si>
-    <t>ilyes_cv.pdf</t>
-  </si>
-  <si>
-    <t>IM</t>
-  </si>
-  <si>
-    <t>CM</t>
-  </si>
-  <si>
-    <t>ING</t>
-  </si>
-  <si>
     <t>active_student</t>
   </si>
   <si>
-    <t>alimeknimekni@gmail.com</t>
-  </si>
-  <si>
-    <t>amineaouidetaouidet@gmail.com</t>
-  </si>
-  <si>
-    <t>amiragafsigafsi@gmail.com</t>
-  </si>
-  <si>
-    <t>islemgafsigafsi@gmail.com</t>
-  </si>
-  <si>
-    <t>ghazinefzinefzi@gmail.com</t>
-  </si>
-  <si>
-    <t>chirazbenboubaker@gmail.com</t>
-  </si>
-  <si>
-    <t>ahmedgafsi88@gmail.com</t>
-  </si>
-  <si>
-    <t>Mzoughi</t>
-  </si>
-  <si>
-    <t>oumaymaamzoughi@gmail.com</t>
-  </si>
-  <si>
-    <t>hafsitsw@gmail.com</t>
+    <t>academicYearlevel</t>
+  </si>
+  <si>
+    <t>1ING</t>
+  </si>
+  <si>
+    <t>aahmedgafsi@gmail.com</t>
+  </si>
+  <si>
+    <t>alimeknimekni123@gmail.com</t>
+  </si>
+  <si>
+    <t>amineaouidet123@gmail.com</t>
+  </si>
+  <si>
+    <t>amiragafsi123@gmail.com</t>
+  </si>
+  <si>
+    <t>islemgafsi123@gmail.com</t>
+  </si>
+  <si>
+    <t>ghazinefzi123@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -624,306 +561,201 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="K1" s="5"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>11526369</v>
+        <v>23456789</v>
       </c>
       <c r="B2" s="2">
         <v>36902</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="F2">
         <v>25234567</v>
       </c>
       <c r="G2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
-      <c r="J2" t="s">
-        <v>38</v>
+        <v>21</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>11526379</v>
+        <v>23456779</v>
       </c>
       <c r="B3" s="2">
         <v>36903</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="F3">
         <v>25234568</v>
       </c>
       <c r="G3" t="s">
-        <v>27</v>
-      </c>
-      <c r="H3" t="s">
-        <v>35</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3" t="s">
-        <v>38</v>
+        <v>21</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>11526389</v>
+        <v>23406789</v>
       </c>
       <c r="B4" s="2">
         <v>36904</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="F4">
         <v>25234579</v>
       </c>
       <c r="G4" t="s">
-        <v>28</v>
-      </c>
-      <c r="H4" t="s">
-        <v>36</v>
-      </c>
-      <c r="I4">
+        <v>21</v>
+      </c>
+      <c r="H4">
         <v>1</v>
       </c>
-      <c r="J4" t="s">
-        <v>38</v>
+      <c r="I4" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>11526399</v>
+        <v>23156789</v>
       </c>
       <c r="B5" s="2">
         <v>36905</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="F5">
         <v>25234581</v>
       </c>
       <c r="G5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I5">
+        <v>21</v>
+      </c>
+      <c r="H5">
         <v>1</v>
       </c>
-      <c r="J5" t="s">
-        <v>38</v>
+      <c r="I5" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>11526319</v>
+        <v>23455789</v>
       </c>
       <c r="B6" s="2">
         <v>36906</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="F6">
         <v>25234582</v>
       </c>
       <c r="G6" t="s">
-        <v>30</v>
-      </c>
-      <c r="H6" t="s">
-        <v>37</v>
-      </c>
-      <c r="I6">
-        <v>2</v>
-      </c>
-      <c r="J6" t="s">
-        <v>38</v>
+        <v>21</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>11526329</v>
+        <v>23477789</v>
       </c>
       <c r="B7" s="2">
         <v>36907</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="F7">
         <v>25234583</v>
       </c>
       <c r="G7" t="s">
-        <v>31</v>
-      </c>
-      <c r="H7" t="s">
-        <v>37</v>
-      </c>
-      <c r="I7">
-        <v>2</v>
-      </c>
-      <c r="J7" t="s">
-        <v>38</v>
+        <v>21</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>11526339</v>
-      </c>
-      <c r="B8" s="2">
-        <v>36908</v>
-      </c>
-      <c r="C8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F8">
-        <v>25234584</v>
-      </c>
-      <c r="G8" t="s">
-        <v>32</v>
-      </c>
-      <c r="H8" t="s">
-        <v>35</v>
-      </c>
-      <c r="I8">
-        <v>3</v>
-      </c>
-      <c r="J8" t="s">
-        <v>38</v>
-      </c>
+      <c r="B8" s="2"/>
+      <c r="E8" s="3"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>11526349</v>
-      </c>
-      <c r="B9" s="2">
-        <v>36909</v>
-      </c>
-      <c r="C9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" t="s">
-        <v>46</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F9">
-        <v>25234585</v>
-      </c>
-      <c r="G9" t="s">
-        <v>33</v>
-      </c>
-      <c r="H9" t="s">
-        <v>35</v>
-      </c>
-      <c r="I9">
-        <v>3</v>
-      </c>
-      <c r="J9" t="s">
-        <v>38</v>
-      </c>
+      <c r="B9" s="2"/>
+      <c r="E9" s="3"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>11526359</v>
-      </c>
-      <c r="B10" s="2">
-        <v>36910</v>
-      </c>
-      <c r="C10" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F10">
-        <v>25234586</v>
-      </c>
-      <c r="G10" t="s">
-        <v>34</v>
-      </c>
-      <c r="H10" t="s">
-        <v>35</v>
-      </c>
-      <c r="I10">
-        <v>3</v>
-      </c>
-      <c r="J10" t="s">
-        <v>38</v>
-      </c>
+      <c r="B10" s="2"/>
+      <c r="E10" s="3"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B11" s="2"/>
@@ -958,14 +790,11 @@
     <hyperlink ref="E2" r:id="rId1" xr:uid="{AC674394-A38F-4CF0-BBCF-1EABECDAE26E}"/>
     <hyperlink ref="E3" r:id="rId2" xr:uid="{2683BA0E-D107-49D1-A535-42A8413C1392}"/>
     <hyperlink ref="E4" r:id="rId3" xr:uid="{ED43BC6E-A0FD-4AAD-B36F-16FFC3B24B7E}"/>
-    <hyperlink ref="E5" r:id="rId4" xr:uid="{FBC6E1C0-2287-4661-95D5-32E3EFAFC6E3}"/>
-    <hyperlink ref="E6" r:id="rId5" xr:uid="{4F197912-C0B7-45BF-9590-4C1BA8176939}"/>
-    <hyperlink ref="E7" r:id="rId6" xr:uid="{DF49EFD0-C932-4EE8-BC93-B7A38DD20FA7}"/>
-    <hyperlink ref="E8" r:id="rId7" xr:uid="{A5057ADE-532C-464A-8B41-755A876B4057}"/>
-    <hyperlink ref="E9" r:id="rId8" xr:uid="{C76FA67C-0334-4551-B9D8-273D708CFC3B}"/>
-    <hyperlink ref="E10" r:id="rId9" xr:uid="{E0FC9139-189A-467A-A089-323F4CC67101}"/>
+    <hyperlink ref="E5" r:id="rId4" xr:uid="{D84D29F8-39EB-4351-86F8-17881FBC6780}"/>
+    <hyperlink ref="E6" r:id="rId5" xr:uid="{590CE1DF-607C-4EFA-8235-667ED9937529}"/>
+    <hyperlink ref="E7" r:id="rId6" xr:uid="{90B03057-7182-436E-A25D-A1C5B43CD38F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId10"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>